<commit_message>
template schedule for finals this semester
</commit_message>
<xml_diff>
--- a/data/course_data3.xlsx
+++ b/data/course_data3.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ercx2\Desktop\Scheduling Theory_02\Paper\scheduling\Campus-Scheduling\data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/9e402f802124af4b/Masaüstü/Projects/Campus-Scheduling/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{12C3B634-61CA-4F04-A71E-C3162BBFCFBF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="3" documentId="13_ncr:1_{12C3B634-61CA-4F04-A71E-C3162BBFCFBF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{CD92768D-85E4-4D92-BD35-7F6AE6BF69CD}"/>
   <bookViews>
-    <workbookView xWindow="-38520" yWindow="5940" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1778" yWindow="1778" windowWidth="16200" windowHeight="9307" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -1404,6 +1404,20 @@
   </cellStyles>
   <dxfs count="3">
     <dxf>
+      <border outline="0">
+        <top style="thin">
+          <color auto="1"/>
+        </top>
+      </border>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <bottom style="thin">
+          <color auto="1"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
       <font>
         <b/>
         <i val="0"/>
@@ -1431,20 +1445,6 @@
         <bottom/>
       </border>
     </dxf>
-    <dxf>
-      <border outline="0">
-        <bottom style="thin">
-          <color auto="1"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <border outline="0">
-        <top style="thin">
-          <color auto="1"/>
-        </top>
-      </border>
-    </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
@@ -1458,9 +1458,19 @@
 </styleSheet>
 </file>
 
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
+</file>
+
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{8A85116F-6A64-4F3C-A7B2-43B3C720AB5E}" name="Table1" displayName="Table1" ref="A1:H232" totalsRowShown="0" headerRowDxfId="0" headerRowBorderDxfId="1" tableBorderDxfId="2">
-  <autoFilter ref="A1:H232" xr:uid="{8A85116F-6A64-4F3C-A7B2-43B3C720AB5E}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{8A85116F-6A64-4F3C-A7B2-43B3C720AB5E}" name="Table1" displayName="Table1" ref="A1:H232" totalsRowShown="0" headerRowDxfId="2" headerRowBorderDxfId="1" tableBorderDxfId="0">
+  <autoFilter ref="A1:H232" xr:uid="{8A85116F-6A64-4F3C-A7B2-43B3C720AB5E}">
+    <filterColumn colId="0">
+      <filters>
+        <filter val="Bilgisayar Mühendisliği"/>
+      </filters>
+    </filterColumn>
+  </autoFilter>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:H232">
     <sortCondition ref="C1:C232"/>
   </sortState>
@@ -1764,17 +1774,17 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:H232"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="1" max="1" width="18.1796875" customWidth="1"/>
-    <col min="2" max="2" width="13.08984375" customWidth="1"/>
-    <col min="3" max="3" width="47.90625" customWidth="1"/>
-    <col min="5" max="5" width="10.26953125" customWidth="1"/>
-    <col min="6" max="6" width="16.6328125" customWidth="1"/>
-    <col min="7" max="7" width="14.1796875" customWidth="1"/>
+    <col min="1" max="1" width="18.19921875" customWidth="1"/>
+    <col min="2" max="2" width="13.06640625" customWidth="1"/>
+    <col min="3" max="3" width="47.9296875" customWidth="1"/>
+    <col min="5" max="5" width="10.265625" customWidth="1"/>
+    <col min="6" max="6" width="16.59765625" customWidth="1"/>
+    <col min="7" max="7" width="14.19921875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1800,7 +1810,7 @@
         <v>439</v>
       </c>
     </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A2" t="s">
         <v>7</v>
       </c>
@@ -1826,7 +1836,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A3" t="s">
         <v>7</v>
       </c>
@@ -1852,7 +1862,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A4" t="s">
         <v>7</v>
       </c>
@@ -1878,7 +1888,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A5" t="s">
         <v>15</v>
       </c>
@@ -1904,7 +1914,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A6" t="s">
         <v>18</v>
       </c>
@@ -1930,7 +1940,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A7" t="s">
         <v>21</v>
       </c>
@@ -1956,7 +1966,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A8" t="s">
         <v>7</v>
       </c>
@@ -1982,7 +1992,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A9" t="s">
         <v>7</v>
       </c>
@@ -2008,7 +2018,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A10" t="s">
         <v>21</v>
       </c>
@@ -2034,7 +2044,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A11" t="s">
         <v>30</v>
       </c>
@@ -2060,7 +2070,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="12" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A12" t="s">
         <v>30</v>
       </c>
@@ -2086,7 +2096,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A13" t="s">
         <v>15</v>
       </c>
@@ -2112,7 +2122,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="14" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A14" t="s">
         <v>37</v>
       </c>
@@ -2138,7 +2148,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="15" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A15" t="s">
         <v>30</v>
       </c>
@@ -2164,7 +2174,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="16" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A16" t="s">
         <v>21</v>
       </c>
@@ -2190,7 +2200,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="17" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A17" t="s">
         <v>37</v>
       </c>
@@ -2216,7 +2226,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="18" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A18" t="s">
         <v>7</v>
       </c>
@@ -2242,7 +2252,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="19" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A19" t="s">
         <v>30</v>
       </c>
@@ -2268,7 +2278,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="20" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A20" t="s">
         <v>21</v>
       </c>
@@ -2294,7 +2304,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="21" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A21" t="s">
         <v>37</v>
       </c>
@@ -2320,7 +2330,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="22" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A22" t="s">
         <v>15</v>
       </c>
@@ -2346,7 +2356,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="23" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A23" t="s">
         <v>30</v>
       </c>
@@ -2372,7 +2382,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="24" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A24" t="s">
         <v>30</v>
       </c>
@@ -2398,7 +2408,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="25" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A25" t="s">
         <v>37</v>
       </c>
@@ -2424,7 +2434,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="26" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A26" t="s">
         <v>7</v>
       </c>
@@ -2450,7 +2460,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="27" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A27" t="s">
         <v>7</v>
       </c>
@@ -2476,7 +2486,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="28" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A28" t="s">
         <v>7</v>
       </c>
@@ -2502,7 +2512,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="29" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A29" t="s">
         <v>18</v>
       </c>
@@ -2528,7 +2538,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="30" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A30" t="s">
         <v>18</v>
       </c>
@@ -2554,7 +2564,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="31" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A31" t="s">
         <v>37</v>
       </c>
@@ -2580,7 +2590,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="32" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A32" t="s">
         <v>30</v>
       </c>
@@ -2606,7 +2616,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="33" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A33" t="s">
         <v>18</v>
       </c>
@@ -2632,7 +2642,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="34" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A34" t="s">
         <v>37</v>
       </c>
@@ -2658,7 +2668,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="35" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A35" t="s">
         <v>37</v>
       </c>
@@ -2684,7 +2694,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="36" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A36" t="s">
         <v>21</v>
       </c>
@@ -2710,7 +2720,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="37" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A37" t="s">
         <v>7</v>
       </c>
@@ -2736,7 +2746,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="38" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A38" t="s">
         <v>30</v>
       </c>
@@ -2762,7 +2772,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="39" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A39" t="s">
         <v>89</v>
       </c>
@@ -2788,7 +2798,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="40" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A40" t="s">
         <v>15</v>
       </c>
@@ -2814,7 +2824,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="41" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A41" t="s">
         <v>37</v>
       </c>
@@ -2840,7 +2850,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="42" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A42" t="s">
         <v>18</v>
       </c>
@@ -2866,7 +2876,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="43" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A43" t="s">
         <v>30</v>
       </c>
@@ -2892,7 +2902,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="44" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A44" t="s">
         <v>15</v>
       </c>
@@ -2918,7 +2928,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="45" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A45" t="s">
         <v>18</v>
       </c>
@@ -2944,7 +2954,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="46" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A46" t="s">
         <v>21</v>
       </c>
@@ -2970,7 +2980,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="47" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A47" t="s">
         <v>37</v>
       </c>
@@ -2996,7 +3006,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="48" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="48" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A48" t="s">
         <v>37</v>
       </c>
@@ -3022,7 +3032,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="49" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="49" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A49" t="s">
         <v>37</v>
       </c>
@@ -3048,7 +3058,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="50" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="50" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A50" t="s">
         <v>37</v>
       </c>
@@ -3074,7 +3084,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="51" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="51" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A51" t="s">
         <v>37</v>
       </c>
@@ -3100,7 +3110,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="52" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="52" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A52" t="s">
         <v>37</v>
       </c>
@@ -3126,7 +3136,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="53" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="53" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A53" t="s">
         <v>37</v>
       </c>
@@ -3152,7 +3162,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="54" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="54" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A54" t="s">
         <v>37</v>
       </c>
@@ -3178,7 +3188,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="55" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="55" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A55" t="s">
         <v>37</v>
       </c>
@@ -3204,7 +3214,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="56" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="56" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A56" t="s">
         <v>21</v>
       </c>
@@ -3230,7 +3240,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="57" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="57" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A57" t="s">
         <v>15</v>
       </c>
@@ -3256,7 +3266,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="58" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="58" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A58" t="s">
         <v>15</v>
       </c>
@@ -3282,7 +3292,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="59" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="59" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A59" t="s">
         <v>18</v>
       </c>
@@ -3308,7 +3318,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="60" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="60" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A60" t="s">
         <v>21</v>
       </c>
@@ -3334,7 +3344,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="61" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="61" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A61" t="s">
         <v>18</v>
       </c>
@@ -3360,7 +3370,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="62" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="62" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A62" t="s">
         <v>7</v>
       </c>
@@ -3386,7 +3396,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="63" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="63" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A63" t="s">
         <v>15</v>
       </c>
@@ -3412,7 +3422,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="64" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="64" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A64" t="s">
         <v>21</v>
       </c>
@@ -3438,7 +3448,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="65" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="65" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A65" t="s">
         <v>15</v>
       </c>
@@ -3464,7 +3474,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="66" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="66" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A66" t="s">
         <v>89</v>
       </c>
@@ -3490,7 +3500,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="67" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="67" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A67" t="s">
         <v>30</v>
       </c>
@@ -3516,7 +3526,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="68" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="68" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A68" t="s">
         <v>21</v>
       </c>
@@ -3542,7 +3552,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="69" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="69" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A69" t="s">
         <v>21</v>
       </c>
@@ -3568,7 +3578,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="70" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="70" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A70" t="s">
         <v>18</v>
       </c>
@@ -3594,7 +3604,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="71" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="71" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A71" t="s">
         <v>37</v>
       </c>
@@ -3620,7 +3630,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="72" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="72" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A72" t="s">
         <v>37</v>
       </c>
@@ -3646,7 +3656,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="73" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="73" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A73" t="s">
         <v>18</v>
       </c>
@@ -3672,7 +3682,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="74" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="74" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A74" t="s">
         <v>18</v>
       </c>
@@ -3698,7 +3708,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="75" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="75" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A75" t="s">
         <v>7</v>
       </c>
@@ -3724,7 +3734,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="76" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="76" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A76" t="s">
         <v>18</v>
       </c>
@@ -3750,7 +3760,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="77" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="77" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A77" t="s">
         <v>18</v>
       </c>
@@ -3776,7 +3786,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="78" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="78" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A78" t="s">
         <v>18</v>
       </c>
@@ -3802,7 +3812,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="79" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="79" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A79" t="s">
         <v>15</v>
       </c>
@@ -3828,7 +3838,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="80" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="80" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A80" t="s">
         <v>89</v>
       </c>
@@ -3854,7 +3864,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="81" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="81" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A81" t="s">
         <v>30</v>
       </c>
@@ -3880,7 +3890,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="82" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="82" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A82" t="s">
         <v>21</v>
       </c>
@@ -3906,7 +3916,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="83" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="83" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A83" t="s">
         <v>21</v>
       </c>
@@ -3932,7 +3942,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="84" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="84" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A84" t="s">
         <v>7</v>
       </c>
@@ -3958,7 +3968,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="85" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="85" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A85" t="s">
         <v>21</v>
       </c>
@@ -3984,7 +3994,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="86" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="86" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A86" t="s">
         <v>21</v>
       </c>
@@ -4010,7 +4020,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="87" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="87" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A87" t="s">
         <v>21</v>
       </c>
@@ -4036,7 +4046,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="88" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="88" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A88" t="s">
         <v>21</v>
       </c>
@@ -4062,7 +4072,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="89" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="89" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A89" t="s">
         <v>21</v>
       </c>
@@ -4088,7 +4098,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="90" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="90" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A90" t="s">
         <v>21</v>
       </c>
@@ -4114,7 +4124,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="91" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="91" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A91" t="s">
         <v>21</v>
       </c>
@@ -4140,7 +4150,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="92" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="92" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A92" t="s">
         <v>21</v>
       </c>
@@ -4166,7 +4176,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="93" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="93" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A93" t="s">
         <v>21</v>
       </c>
@@ -4192,7 +4202,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="94" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="94" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A94" t="s">
         <v>21</v>
       </c>
@@ -4218,7 +4228,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="95" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="95" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A95" t="s">
         <v>15</v>
       </c>
@@ -4244,7 +4254,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="96" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="96" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A96" t="s">
         <v>30</v>
       </c>
@@ -4270,7 +4280,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="97" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="97" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A97" t="s">
         <v>15</v>
       </c>
@@ -4296,7 +4306,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="98" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="98" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A98" t="s">
         <v>30</v>
       </c>
@@ -4322,7 +4332,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="99" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="99" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A99" t="s">
         <v>15</v>
       </c>
@@ -4348,7 +4358,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="100" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="100" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A100" t="s">
         <v>37</v>
       </c>
@@ -4374,7 +4384,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="101" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="101" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A101" t="s">
         <v>37</v>
       </c>
@@ -4400,7 +4410,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="102" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="102" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A102" t="s">
         <v>15</v>
       </c>
@@ -4426,7 +4436,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="103" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="103" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A103" t="s">
         <v>15</v>
       </c>
@@ -4452,7 +4462,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="104" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="104" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A104" t="s">
         <v>30</v>
       </c>
@@ -4478,7 +4488,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="105" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="105" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A105" t="s">
         <v>30</v>
       </c>
@@ -4504,7 +4514,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="106" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="106" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A106" t="s">
         <v>18</v>
       </c>
@@ -4530,7 +4540,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="107" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="107" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A107" t="s">
         <v>18</v>
       </c>
@@ -4556,7 +4566,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="108" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="108" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A108" t="s">
         <v>37</v>
       </c>
@@ -4582,7 +4592,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="109" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="109" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A109" t="s">
         <v>7</v>
       </c>
@@ -4608,7 +4618,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="110" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="110" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A110" t="s">
         <v>18</v>
       </c>
@@ -4634,7 +4644,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="111" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="111" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A111" t="s">
         <v>18</v>
       </c>
@@ -4660,7 +4670,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="112" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="112" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A112" t="s">
         <v>30</v>
       </c>
@@ -4686,7 +4696,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="113" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="113" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A113" t="s">
         <v>15</v>
       </c>
@@ -4712,7 +4722,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="114" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="114" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A114" t="s">
         <v>37</v>
       </c>
@@ -4738,7 +4748,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="115" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="115" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A115" t="s">
         <v>21</v>
       </c>
@@ -4764,7 +4774,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="116" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="116" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A116" t="s">
         <v>15</v>
       </c>
@@ -4790,7 +4800,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="117" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="117" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A117" t="s">
         <v>89</v>
       </c>
@@ -4816,7 +4826,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="118" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="118" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A118" t="s">
         <v>89</v>
       </c>
@@ -4842,7 +4852,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="119" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="119" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A119" t="s">
         <v>15</v>
       </c>
@@ -4868,7 +4878,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="120" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="120" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A120" t="s">
         <v>15</v>
       </c>
@@ -4894,7 +4904,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="121" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="121" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A121" t="s">
         <v>30</v>
       </c>
@@ -4920,7 +4930,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="122" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="122" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A122" t="s">
         <v>30</v>
       </c>
@@ -4946,7 +4956,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="123" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="123" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A123" t="s">
         <v>7</v>
       </c>
@@ -4972,7 +4982,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="124" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="124" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A124" t="s">
         <v>89</v>
       </c>
@@ -4998,7 +5008,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="125" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="125" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A125" t="s">
         <v>89</v>
       </c>
@@ -5024,7 +5034,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="126" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="126" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A126" t="s">
         <v>15</v>
       </c>
@@ -5050,7 +5060,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="127" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="127" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A127" t="s">
         <v>7</v>
       </c>
@@ -5076,7 +5086,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="128" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="128" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A128" t="s">
         <v>30</v>
       </c>
@@ -5102,7 +5112,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="129" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="129" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A129" t="s">
         <v>89</v>
       </c>
@@ -5128,7 +5138,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="130" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="130" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A130" t="s">
         <v>15</v>
       </c>
@@ -5154,7 +5164,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="131" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="131" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A131" t="s">
         <v>89</v>
       </c>
@@ -5180,7 +5190,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="132" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="132" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A132" t="s">
         <v>21</v>
       </c>
@@ -5206,7 +5216,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="133" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="133" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A133" t="s">
         <v>21</v>
       </c>
@@ -5232,7 +5242,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="134" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="134" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A134" t="s">
         <v>89</v>
       </c>
@@ -5258,7 +5268,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="135" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="135" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A135" t="s">
         <v>15</v>
       </c>
@@ -5284,7 +5294,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="136" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="136" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A136" t="s">
         <v>15</v>
       </c>
@@ -5310,7 +5320,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="137" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="137" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A137" t="s">
         <v>15</v>
       </c>
@@ -5336,7 +5346,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="138" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="138" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A138" t="s">
         <v>15</v>
       </c>
@@ -5362,7 +5372,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="139" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="139" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A139" t="s">
         <v>15</v>
       </c>
@@ -5388,7 +5398,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="140" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="140" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A140" t="s">
         <v>30</v>
       </c>
@@ -5414,7 +5424,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="141" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="141" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A141" t="s">
         <v>37</v>
       </c>
@@ -5440,7 +5450,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="142" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="142" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A142" t="s">
         <v>37</v>
       </c>
@@ -5466,7 +5476,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="143" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="143" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A143" t="s">
         <v>89</v>
       </c>
@@ -5492,7 +5502,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="144" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="144" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A144" t="s">
         <v>30</v>
       </c>
@@ -5518,7 +5528,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="145" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="145" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A145" t="s">
         <v>21</v>
       </c>
@@ -5544,7 +5554,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="146" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="146" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A146" t="s">
         <v>15</v>
       </c>
@@ -5570,7 +5580,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="147" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="147" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A147" t="s">
         <v>18</v>
       </c>
@@ -5596,7 +5606,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="148" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="148" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A148" t="s">
         <v>7</v>
       </c>
@@ -5622,7 +5632,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="149" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="149" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A149" t="s">
         <v>37</v>
       </c>
@@ -5648,7 +5658,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="150" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="150" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A150" t="s">
         <v>15</v>
       </c>
@@ -5674,7 +5684,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="151" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="151" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A151" t="s">
         <v>15</v>
       </c>
@@ -5700,7 +5710,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="152" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="152" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A152" t="s">
         <v>7</v>
       </c>
@@ -5726,7 +5736,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="153" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="153" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A153" t="s">
         <v>89</v>
       </c>
@@ -5752,7 +5762,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="154" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="154" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A154" t="s">
         <v>21</v>
       </c>
@@ -5778,7 +5788,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="155" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="155" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A155" t="s">
         <v>21</v>
       </c>
@@ -5804,7 +5814,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="156" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="156" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A156" t="s">
         <v>18</v>
       </c>
@@ -5830,7 +5840,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="157" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="157" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A157" t="s">
         <v>21</v>
       </c>
@@ -5856,7 +5866,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="158" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="158" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A158" t="s">
         <v>21</v>
       </c>
@@ -5882,7 +5892,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="159" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="159" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A159" t="s">
         <v>89</v>
       </c>
@@ -5908,7 +5918,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="160" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="160" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A160" t="s">
         <v>37</v>
       </c>
@@ -5934,7 +5944,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="161" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="161" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A161" t="s">
         <v>37</v>
       </c>
@@ -5960,7 +5970,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="162" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="162" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A162" t="s">
         <v>89</v>
       </c>
@@ -5986,7 +5996,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="163" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="163" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A163" t="s">
         <v>30</v>
       </c>
@@ -6012,7 +6022,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="164" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="164" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A164" t="s">
         <v>15</v>
       </c>
@@ -6038,7 +6048,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="165" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="165" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A165" t="s">
         <v>18</v>
       </c>
@@ -6064,7 +6074,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="166" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="166" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A166" t="s">
         <v>18</v>
       </c>
@@ -6090,7 +6100,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="167" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="167" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A167" t="s">
         <v>7</v>
       </c>
@@ -6116,7 +6126,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="168" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="168" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A168" t="s">
         <v>7</v>
       </c>
@@ -6142,7 +6152,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="169" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="169" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A169" t="s">
         <v>30</v>
       </c>
@@ -6168,7 +6178,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="170" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="170" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A170" t="s">
         <v>15</v>
       </c>
@@ -6194,7 +6204,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="171" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="171" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A171" t="s">
         <v>89</v>
       </c>
@@ -6220,7 +6230,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="172" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="172" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A172" t="s">
         <v>15</v>
       </c>
@@ -6246,7 +6256,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="173" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="173" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A173" t="s">
         <v>37</v>
       </c>
@@ -6272,7 +6282,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="174" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="174" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A174" t="s">
         <v>37</v>
       </c>
@@ -6298,7 +6308,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="175" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="175" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A175" t="s">
         <v>89</v>
       </c>
@@ -6324,7 +6334,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="176" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="176" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A176" t="s">
         <v>7</v>
       </c>
@@ -6350,7 +6360,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="177" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="177" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A177" t="s">
         <v>18</v>
       </c>
@@ -6376,7 +6386,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="178" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="178" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A178" t="s">
         <v>7</v>
       </c>
@@ -6402,7 +6412,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="179" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="179" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A179" t="s">
         <v>37</v>
       </c>
@@ -6428,7 +6438,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="180" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="180" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A180" t="s">
         <v>30</v>
       </c>
@@ -6454,7 +6464,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="181" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="181" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A181" t="s">
         <v>37</v>
       </c>
@@ -6480,7 +6490,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="182" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="182" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A182" t="s">
         <v>37</v>
       </c>
@@ -6506,7 +6516,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="183" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="183" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A183" t="s">
         <v>37</v>
       </c>
@@ -6532,7 +6542,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="184" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="184" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A184" t="s">
         <v>18</v>
       </c>
@@ -6558,7 +6568,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="185" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="185" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A185" t="s">
         <v>37</v>
       </c>
@@ -6584,7 +6594,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="186" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="186" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A186" t="s">
         <v>15</v>
       </c>
@@ -6610,7 +6620,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="187" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="187" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A187" t="s">
         <v>15</v>
       </c>
@@ -6636,7 +6646,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="188" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="188" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A188" t="s">
         <v>30</v>
       </c>
@@ -6662,7 +6672,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="189" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="189" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A189" t="s">
         <v>89</v>
       </c>
@@ -6688,7 +6698,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="190" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="190" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A190" t="s">
         <v>89</v>
       </c>
@@ -6714,7 +6724,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="191" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="191" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A191" t="s">
         <v>21</v>
       </c>
@@ -6740,7 +6750,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="192" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="192" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A192" t="s">
         <v>37</v>
       </c>
@@ -6766,7 +6776,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="193" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="193" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A193" t="s">
         <v>15</v>
       </c>
@@ -6792,7 +6802,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="194" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="194" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A194" t="s">
         <v>15</v>
       </c>
@@ -6818,7 +6828,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="195" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="195" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A195" t="s">
         <v>89</v>
       </c>
@@ -6844,7 +6854,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="196" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="196" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A196" t="s">
         <v>18</v>
       </c>
@@ -6870,7 +6880,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="197" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="197" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A197" t="s">
         <v>7</v>
       </c>
@@ -6896,7 +6906,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="198" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="198" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A198" t="s">
         <v>7</v>
       </c>
@@ -6922,7 +6932,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="199" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="199" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A199" t="s">
         <v>30</v>
       </c>
@@ -6948,7 +6958,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="200" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="200" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A200" t="s">
         <v>21</v>
       </c>
@@ -6974,7 +6984,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="201" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="201" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A201" t="s">
         <v>15</v>
       </c>
@@ -7000,7 +7010,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="202" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="202" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A202" t="s">
         <v>15</v>
       </c>
@@ -7026,7 +7036,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="203" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="203" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A203" t="s">
         <v>7</v>
       </c>
@@ -7052,7 +7062,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="204" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="204" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A204" t="s">
         <v>21</v>
       </c>
@@ -7078,7 +7088,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="205" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="205" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A205" t="s">
         <v>15</v>
       </c>
@@ -7104,7 +7114,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="206" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="206" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A206" t="s">
         <v>15</v>
       </c>
@@ -7130,7 +7140,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="207" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="207" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A207" t="s">
         <v>7</v>
       </c>
@@ -7156,7 +7166,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="208" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="208" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A208" t="s">
         <v>15</v>
       </c>
@@ -7182,7 +7192,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="209" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="209" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A209" t="s">
         <v>30</v>
       </c>
@@ -7208,7 +7218,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="210" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="210" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A210" t="s">
         <v>89</v>
       </c>
@@ -7234,7 +7244,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="211" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="211" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A211" t="s">
         <v>21</v>
       </c>
@@ -7260,7 +7270,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="212" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="212" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A212" t="s">
         <v>30</v>
       </c>
@@ -7286,7 +7296,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="213" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="213" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A213" t="s">
         <v>21</v>
       </c>
@@ -7312,7 +7322,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="214" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="214" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A214" t="s">
         <v>7</v>
       </c>
@@ -7338,7 +7348,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="215" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="215" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A215" t="s">
         <v>15</v>
       </c>
@@ -7364,7 +7374,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="216" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="216" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A216" t="s">
         <v>7</v>
       </c>
@@ -7390,7 +7400,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="217" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="217" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A217" t="s">
         <v>15</v>
       </c>
@@ -7416,7 +7426,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="218" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="218" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A218" t="s">
         <v>89</v>
       </c>
@@ -7442,7 +7452,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="219" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="219" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A219" t="s">
         <v>30</v>
       </c>
@@ -7468,7 +7478,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="220" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="220" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A220" t="s">
         <v>89</v>
       </c>
@@ -7494,7 +7504,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="221" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="221" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A221" t="s">
         <v>89</v>
       </c>
@@ -7520,7 +7530,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="222" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="222" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A222" t="s">
         <v>18</v>
       </c>
@@ -7546,7 +7556,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="223" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="223" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A223" t="s">
         <v>15</v>
       </c>
@@ -7572,7 +7582,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="224" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="224" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A224" t="s">
         <v>30</v>
       </c>
@@ -7598,7 +7608,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="225" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="225" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A225" t="s">
         <v>30</v>
       </c>
@@ -7624,7 +7634,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="226" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="226" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A226" t="s">
         <v>30</v>
       </c>
@@ -7650,7 +7660,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="227" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="227" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A227" t="s">
         <v>30</v>
       </c>
@@ -7676,7 +7686,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="228" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="228" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A228" t="s">
         <v>30</v>
       </c>
@@ -7702,7 +7712,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="229" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="229" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A229" t="s">
         <v>89</v>
       </c>
@@ -7728,7 +7738,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="230" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="230" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A230" t="s">
         <v>37</v>
       </c>
@@ -7754,7 +7764,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="231" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="231" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A231" t="s">
         <v>15</v>
       </c>
@@ -7780,7 +7790,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="232" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="232" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A232" t="s">
         <v>30</v>
       </c>

</xml_diff>